<commit_message>
GLOB-896: The premium and tax calculation for cancellations was adjusted to consider all policy transactions and apply the corresponding prorated calculation to each one.
</commit_message>
<xml_diff>
--- a/Documentación/calculo de endoso de cancelacion.xlsx
+++ b/Documentación/calculo de endoso de cancelacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Global\Documentación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C41617BC-F68E-4893-8868-7AEB92B3CD6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2DA1DA1-2060-48E1-95C5-D48D8248985B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{29E951A4-280C-4344-B043-AA9C6C8BBF6F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="18">
   <si>
     <t>emision</t>
   </si>
@@ -90,6 +90,9 @@
   </si>
   <si>
     <t>Cancelación de la disminución</t>
+  </si>
+  <si>
+    <t>Montos a cancelar</t>
   </si>
 </sst>
 </file>
@@ -99,7 +102,7 @@
   <numFmts count="1">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -122,13 +125,27 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -144,16 +161,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Millares" xfId="1" builtinId="3"/>
@@ -581,7 +604,7 @@
         <f>+B11+E11</f>
         <v>4.07</v>
       </c>
-      <c r="H11" s="6"/>
+      <c r="H11" s="5"/>
       <c r="K11" s="1">
         <v>46388</v>
       </c>
@@ -607,17 +630,17 @@
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="5" t="s">
+      <c r="A14" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="5"/>
-      <c r="D14" s="5" t="s">
+      <c r="B14" s="6"/>
+      <c r="D14" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="5"/>
-      <c r="F14" s="5"/>
-      <c r="G14" s="5"/>
-      <c r="H14" s="5"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="6"/>
+      <c r="H14" s="6"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
@@ -650,7 +673,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>7</v>
       </c>
@@ -670,7 +693,13 @@
         <v>0.64071856287425155</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="G18" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H18" s="7"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>8</v>
       </c>
@@ -685,12 +714,13 @@
         <f>ROUND((E10/E12)*E17,2)</f>
         <v>-43.97</v>
       </c>
-      <c r="F19">
+      <c r="G19" s="8">
         <f>+B19+E19</f>
         <v>43.980000000000004</v>
       </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H19" s="8"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>10</v>
       </c>
@@ -705,12 +735,13 @@
         <f>ROUND(E19*5%,2)</f>
         <v>-2.2000000000000002</v>
       </c>
-      <c r="F20">
+      <c r="G20" s="8">
         <f>+B20+E20</f>
         <v>2.2000000000000002</v>
       </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H20" s="8"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>14</v>
       </c>
@@ -721,27 +752,32 @@
       <c r="D21" t="s">
         <v>14</v>
       </c>
-      <c r="F21">
-        <f>SUM(F19:F20)</f>
+      <c r="G21" s="8">
+        <f>SUM(G19:G20)</f>
         <v>46.180000000000007</v>
       </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="H21" s="8"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B22">
         <f>+B20+E20</f>
         <v>2.2000000000000002</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B23">
         <f>SUM(B21:B22)</f>
         <v>46.180000000000007</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="6">
+    <mergeCell ref="G21:H21"/>
     <mergeCell ref="D14:H14"/>
     <mergeCell ref="A14:B14"/>
+    <mergeCell ref="G18:H18"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="G20:H20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -749,23 +785,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="d7a6abae-64b1-4e63-a306-b9d1c75aa12c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101000CAD9BF665BEF34DA130572F59E9FB02" ma:contentTypeVersion="9" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="13294a8e09781d8c6dc685cc36271987">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="d7a6abae-64b1-4e63-a306-b9d1c75aa12c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="34159b3cc2126f72f2bfa9841dbaa51f" ns3:_="">
     <xsd:import namespace="d7a6abae-64b1-4e63-a306-b9d1c75aa12c"/>
@@ -941,10 +960,37 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="d7a6abae-64b1-4e63-a306-b9d1c75aa12c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9763EFCA-81E8-4A37-9FD0-D6B2CCC39C20}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1FFA3D5-3D1B-46C7-AF8C-72D349A58D64}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="d7a6abae-64b1-4e63-a306-b9d1c75aa12c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -966,19 +1012,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1FFA3D5-3D1B-46C7-AF8C-72D349A58D64}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9763EFCA-81E8-4A37-9FD0-D6B2CCC39C20}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="d7a6abae-64b1-4e63-a306-b9d1c75aa12c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
GLOB-944: Adjustments were made to the cancellation process related to endorsement detail calculations and the presentation of policy balance information. The endorsement generation process was also updated.
</commit_message>
<xml_diff>
--- a/Documentación/calculo de endoso de cancelacion.xlsx
+++ b/Documentación/calculo de endoso de cancelacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Global\Documentación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2DA1DA1-2060-48E1-95C5-D48D8248985B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ACB0D29-3132-4E6F-A234-2EBB9DEBD6DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{29E951A4-280C-4344-B043-AA9C6C8BBF6F}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="19">
   <si>
     <t>emision</t>
   </si>
@@ -93,6 +93,9 @@
   </si>
   <si>
     <t>Montos a cancelar</t>
+  </si>
+  <si>
+    <t>Saldo Devengado</t>
   </si>
 </sst>
 </file>
@@ -168,14 +171,14 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="43" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="3" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -497,6 +500,7 @@
   <cols>
     <col min="1" max="1" width="25" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="26" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="16.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -506,19 +510,23 @@
       <c r="D6" s="2" t="s">
         <v>13</v>
       </c>
+      <c r="F6">
+        <v>95000</v>
+      </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="3">
-        <v>100000</v>
+        <v>78500</v>
       </c>
       <c r="D7" t="s">
         <v>12</v>
       </c>
       <c r="E7" s="3">
-        <v>-50000</v>
+        <f>+F6-B7</f>
+        <v>16500</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -526,17 +534,17 @@
         <v>1</v>
       </c>
       <c r="B8" s="1">
-        <v>46023</v>
+        <v>46082</v>
       </c>
       <c r="D8" t="s">
         <v>1</v>
       </c>
       <c r="E8" s="1">
-        <v>46054</v>
+        <v>46174</v>
       </c>
       <c r="F8">
         <f>+E7/B7</f>
-        <v>-0.5</v>
+        <v>0.21019108280254778</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -544,21 +552,21 @@
         <v>2</v>
       </c>
       <c r="B9" s="1">
-        <v>46388</v>
+        <v>46447</v>
       </c>
       <c r="D9" t="s">
         <v>2</v>
       </c>
       <c r="E9" s="1">
-        <v>46388</v>
+        <v>46447</v>
       </c>
       <c r="F9" s="4">
         <f>+E9-E8</f>
-        <v>334</v>
+        <v>273</v>
       </c>
       <c r="G9">
         <f>+F9/365</f>
-        <v>0.91506849315068495</v>
+        <v>0.74794520547945209</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -566,22 +574,22 @@
         <v>3</v>
       </c>
       <c r="B10" s="3">
-        <v>150</v>
+        <v>117.75</v>
       </c>
       <c r="D10" t="s">
         <v>3</v>
       </c>
       <c r="E10" s="3">
         <f>+ROUND( F10*G9,2)</f>
-        <v>-68.63</v>
+        <v>18.510000000000002</v>
       </c>
       <c r="F10">
         <f>+F8*B10</f>
-        <v>-75</v>
+        <v>24.75</v>
       </c>
       <c r="G10" s="3">
         <f>+B10+E10</f>
-        <v>81.37</v>
+        <v>136.26</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -589,20 +597,20 @@
         <v>9</v>
       </c>
       <c r="B11">
-        <f>B10*5%</f>
-        <v>7.5</v>
+        <f>ROUND( B10*5%,2)</f>
+        <v>5.89</v>
       </c>
       <c r="D11" t="s">
         <v>9</v>
       </c>
       <c r="E11">
         <f>ROUND(E10*5%,2)</f>
-        <v>-3.43</v>
+        <v>0.93</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="4">
         <f>+B11+E11</f>
-        <v>4.07</v>
+        <v>6.8199999999999994</v>
       </c>
       <c r="H11" s="5"/>
       <c r="K11" s="1">
@@ -622,39 +630,39 @@
       </c>
       <c r="E12">
         <f>E9-E8</f>
-        <v>334</v>
+        <v>273</v>
       </c>
       <c r="G12" s="3">
         <f>SUM(G10:G11)</f>
-        <v>85.44</v>
+        <v>143.07999999999998</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="6"/>
-      <c r="D14" s="6" t="s">
+      <c r="B14" s="7"/>
+      <c r="D14" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
+      <c r="H14" s="7"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>5</v>
       </c>
       <c r="B15" s="1">
-        <v>46174</v>
+        <v>46219</v>
       </c>
       <c r="D15" t="s">
         <v>5</v>
       </c>
       <c r="E15" s="1">
         <f>B15</f>
-        <v>46174</v>
+        <v>46219</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -663,111 +671,130 @@
       </c>
       <c r="B16">
         <f>B15-B8</f>
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="D16" t="s">
         <v>6</v>
       </c>
       <c r="E16">
         <f>E15-E8</f>
-        <v>120</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>7</v>
       </c>
       <c r="B17">
         <f>B9-B15</f>
-        <v>214</v>
+        <v>228</v>
       </c>
       <c r="D17" t="s">
         <v>7</v>
       </c>
       <c r="E17">
         <f>E9-E15</f>
-        <v>214</v>
+        <v>228</v>
       </c>
       <c r="F17">
         <f>+E17/E12</f>
-        <v>0.64071856287425155</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="G18" s="7" t="s">
+        <v>0.8351648351648352</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="G18" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H18" s="7"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="H18" s="8"/>
+      <c r="I18" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>8</v>
       </c>
       <c r="B19">
         <f>ROUND((B10/B12)*B17,2)</f>
-        <v>87.95</v>
+        <v>73.55</v>
       </c>
       <c r="D19" t="s">
         <v>8</v>
       </c>
       <c r="E19">
         <f>ROUND((E10/E12)*E17,2)</f>
-        <v>-43.97</v>
-      </c>
-      <c r="G19" s="8">
+        <v>15.46</v>
+      </c>
+      <c r="G19" s="6">
         <f>+B19+E19</f>
-        <v>43.980000000000004</v>
-      </c>
-      <c r="H19" s="8"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+        <v>89.009999999999991</v>
+      </c>
+      <c r="H19" s="6"/>
+      <c r="I19" s="5">
+        <f>+G10-G19</f>
+        <v>47.25</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>10</v>
       </c>
       <c r="B20">
         <f>ROUND(B19*5%,2)</f>
-        <v>4.4000000000000004</v>
+        <v>3.68</v>
       </c>
       <c r="D20" t="s">
         <v>10</v>
       </c>
       <c r="E20">
         <f>ROUND(E19*5%,2)</f>
-        <v>-2.2000000000000002</v>
-      </c>
-      <c r="G20" s="8">
+        <v>0.77</v>
+      </c>
+      <c r="G20" s="6">
         <f>+B20+E20</f>
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="H20" s="8"/>
-    </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+        <v>4.45</v>
+      </c>
+      <c r="H20" s="6"/>
+      <c r="I20" s="5">
+        <f>+G11-G20</f>
+        <v>2.3699999999999992</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>14</v>
       </c>
       <c r="B21">
         <f>+B19+E19</f>
-        <v>43.980000000000004</v>
+        <v>89.009999999999991</v>
       </c>
       <c r="D21" t="s">
         <v>14</v>
       </c>
-      <c r="G21" s="8">
+      <c r="E21">
+        <f>+E19+E20</f>
+        <v>16.23</v>
+      </c>
+      <c r="G21" s="6">
         <f>SUM(G19:G20)</f>
-        <v>46.180000000000007</v>
-      </c>
-      <c r="H21" s="8"/>
-    </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+        <v>93.46</v>
+      </c>
+      <c r="H21" s="6"/>
+      <c r="I21" s="5">
+        <f>+G12-G21</f>
+        <v>49.61999999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B22">
         <f>+B20+E20</f>
-        <v>2.2000000000000002</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+        <v>4.45</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B23">
         <f>SUM(B21:B22)</f>
-        <v>46.180000000000007</v>
+        <v>93.46</v>
       </c>
     </row>
   </sheetData>
@@ -785,6 +812,23 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="d7a6abae-64b1-4e63-a306-b9d1c75aa12c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x0101000CAD9BF665BEF34DA130572F59E9FB02" ma:contentTypeVersion="9" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="13294a8e09781d8c6dc685cc36271987">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="d7a6abae-64b1-4e63-a306-b9d1c75aa12c" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="34159b3cc2126f72f2bfa9841dbaa51f" ns3:_="">
     <xsd:import namespace="d7a6abae-64b1-4e63-a306-b9d1c75aa12c"/>
@@ -960,37 +1004,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="d7a6abae-64b1-4e63-a306-b9d1c75aa12c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1FFA3D5-3D1B-46C7-AF8C-72D349A58D64}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9763EFCA-81E8-4A37-9FD0-D6B2CCC39C20}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="d7a6abae-64b1-4e63-a306-b9d1c75aa12c"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -1012,9 +1029,19 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9763EFCA-81E8-4A37-9FD0-D6B2CCC39C20}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D1FFA3D5-3D1B-46C7-AF8C-72D349A58D64}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="d7a6abae-64b1-4e63-a306-b9d1c75aa12c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Ajustes cálculos cambio de objeto asegurado
</commit_message>
<xml_diff>
--- a/Documentación/calculo de endoso de cancelacion.xlsx
+++ b/Documentación/calculo de endoso de cancelacion.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Global\Documentación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3ACB0D29-3132-4E6F-A234-2EBB9DEBD6DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A7D967C-C853-4900-824A-C656FEF915DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{29E951A4-280C-4344-B043-AA9C6C8BBF6F}"/>
   </bookViews>
@@ -519,14 +519,13 @@
         <v>11</v>
       </c>
       <c r="B7" s="3">
-        <v>78500</v>
+        <v>40000</v>
       </c>
       <c r="D7" t="s">
         <v>12</v>
       </c>
       <c r="E7" s="3">
-        <f>+F6-B7</f>
-        <v>16500</v>
+        <v>-10000</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
@@ -534,17 +533,17 @@
         <v>1</v>
       </c>
       <c r="B8" s="1">
-        <v>46082</v>
+        <v>46174</v>
       </c>
       <c r="D8" t="s">
         <v>1</v>
       </c>
       <c r="E8" s="1">
-        <v>46174</v>
+        <v>46246</v>
       </c>
       <c r="F8">
         <f>+E7/B7</f>
-        <v>0.21019108280254778</v>
+        <v>-0.25</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -552,21 +551,21 @@
         <v>2</v>
       </c>
       <c r="B9" s="1">
-        <v>46447</v>
+        <v>46539</v>
       </c>
       <c r="D9" t="s">
         <v>2</v>
       </c>
       <c r="E9" s="1">
-        <v>46447</v>
+        <v>46539</v>
       </c>
       <c r="F9" s="4">
         <f>+E9-E8</f>
-        <v>273</v>
+        <v>293</v>
       </c>
       <c r="G9">
         <f>+F9/365</f>
-        <v>0.74794520547945209</v>
+        <v>0.80273972602739729</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -574,22 +573,22 @@
         <v>3</v>
       </c>
       <c r="B10" s="3">
-        <v>117.75</v>
+        <v>180</v>
       </c>
       <c r="D10" t="s">
         <v>3</v>
       </c>
       <c r="E10" s="3">
         <f>+ROUND( F10*G9,2)</f>
-        <v>18.510000000000002</v>
+        <v>-36.119999999999997</v>
       </c>
       <c r="F10">
         <f>+F8*B10</f>
-        <v>24.75</v>
+        <v>-45</v>
       </c>
       <c r="G10" s="3">
         <f>+B10+E10</f>
-        <v>136.26</v>
+        <v>143.88</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -598,19 +597,19 @@
       </c>
       <c r="B11">
         <f>ROUND( B10*5%,2)</f>
-        <v>5.89</v>
+        <v>9</v>
       </c>
       <c r="D11" t="s">
         <v>9</v>
       </c>
       <c r="E11">
         <f>ROUND(E10*5%,2)</f>
-        <v>0.93</v>
+        <v>-1.81</v>
       </c>
       <c r="F11" s="3"/>
       <c r="G11" s="4">
         <f>+B11+E11</f>
-        <v>6.8199999999999994</v>
+        <v>7.1899999999999995</v>
       </c>
       <c r="H11" s="5"/>
       <c r="K11" s="1">
@@ -630,11 +629,11 @@
       </c>
       <c r="E12">
         <f>E9-E8</f>
-        <v>273</v>
+        <v>293</v>
       </c>
       <c r="G12" s="3">
         <f>SUM(G10:G11)</f>
-        <v>143.07999999999998</v>
+        <v>151.07</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -671,14 +670,14 @@
       </c>
       <c r="B16">
         <f>B15-B8</f>
-        <v>137</v>
+        <v>45</v>
       </c>
       <c r="D16" t="s">
         <v>6</v>
       </c>
       <c r="E16">
         <f>E15-E8</f>
-        <v>45</v>
+        <v>-27</v>
       </c>
     </row>
     <row r="17" spans="1:9" x14ac:dyDescent="0.25">
@@ -687,18 +686,18 @@
       </c>
       <c r="B17">
         <f>B9-B15</f>
-        <v>228</v>
+        <v>320</v>
       </c>
       <c r="D17" t="s">
         <v>7</v>
       </c>
       <c r="E17">
         <f>E9-E15</f>
-        <v>228</v>
+        <v>320</v>
       </c>
       <c r="F17">
         <f>+E17/E12</f>
-        <v>0.8351648351648352</v>
+        <v>1.0921501706484642</v>
       </c>
     </row>
     <row r="18" spans="1:9" x14ac:dyDescent="0.25">
@@ -716,23 +715,23 @@
       </c>
       <c r="B19">
         <f>ROUND((B10/B12)*B17,2)</f>
-        <v>73.55</v>
+        <v>157.81</v>
       </c>
       <c r="D19" t="s">
         <v>8</v>
       </c>
       <c r="E19">
         <f>ROUND((E10/E12)*E17,2)</f>
-        <v>15.46</v>
+        <v>-39.450000000000003</v>
       </c>
       <c r="G19" s="6">
         <f>+B19+E19</f>
-        <v>89.009999999999991</v>
+        <v>118.36</v>
       </c>
       <c r="H19" s="6"/>
       <c r="I19" s="5">
         <f>+G10-G19</f>
-        <v>47.25</v>
+        <v>25.519999999999996</v>
       </c>
     </row>
     <row r="20" spans="1:9" x14ac:dyDescent="0.25">
@@ -741,23 +740,23 @@
       </c>
       <c r="B20">
         <f>ROUND(B19*5%,2)</f>
-        <v>3.68</v>
+        <v>7.89</v>
       </c>
       <c r="D20" t="s">
         <v>10</v>
       </c>
       <c r="E20">
         <f>ROUND(E19*5%,2)</f>
-        <v>0.77</v>
+        <v>-1.97</v>
       </c>
       <c r="G20" s="6">
         <f>+B20+E20</f>
-        <v>4.45</v>
+        <v>5.92</v>
       </c>
       <c r="H20" s="6"/>
       <c r="I20" s="5">
         <f>+G11-G20</f>
-        <v>2.3699999999999992</v>
+        <v>1.2699999999999996</v>
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
@@ -766,35 +765,35 @@
       </c>
       <c r="B21">
         <f>+B19+E19</f>
-        <v>89.009999999999991</v>
+        <v>118.36</v>
       </c>
       <c r="D21" t="s">
         <v>14</v>
       </c>
       <c r="E21">
         <f>+E19+E20</f>
-        <v>16.23</v>
+        <v>-41.42</v>
       </c>
       <c r="G21" s="6">
         <f>SUM(G19:G20)</f>
-        <v>93.46</v>
+        <v>124.28</v>
       </c>
       <c r="H21" s="6"/>
       <c r="I21" s="5">
         <f>+G12-G21</f>
-        <v>49.61999999999999</v>
+        <v>26.789999999999992</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B22">
         <f>+B20+E20</f>
-        <v>4.45</v>
+        <v>5.92</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B23">
         <f>SUM(B21:B22)</f>
-        <v>93.46</v>
+        <v>124.28</v>
       </c>
     </row>
   </sheetData>
@@ -812,20 +811,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="d7a6abae-64b1-4e63-a306-b9d1c75aa12c" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="d7a6abae-64b1-4e63-a306-b9d1c75aa12c" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1005,14 +1004,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9763EFCA-81E8-4A37-9FD0-D6B2CCC39C20}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{034CE750-A111-45CE-B135-8E7C0A55A939}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
@@ -1024,6 +1015,14 @@
     <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
     <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9763EFCA-81E8-4A37-9FD0-D6B2CCC39C20}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>